<commit_message>
final of this branch
</commit_message>
<xml_diff>
--- a/Credentials/Credentials.xlsx
+++ b/Credentials/Credentials.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="2" r:id="rId1"/>
@@ -159,10 +159,10 @@
     <t>target query</t>
   </si>
   <si>
+    <t>SELECT empid,  name FROM employees where name != "prashant"</t>
+  </si>
+  <si>
     <t>SELECT * FROM employees</t>
-  </si>
-  <si>
-    <t>SELECT empid,  name FROM employees where name != "prashant"</t>
   </si>
 </sst>
 </file>
@@ -808,10 +808,10 @@
         <v>33</v>
       </c>
       <c r="E5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" t="s">
         <v>46</v>
-      </c>
-      <c r="F5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">

</xml_diff>